<commit_message>
Fix listing copy rules and split operations deliverables
</commit_message>
<xml_diff>
--- a/plugins/chenyu-yunying/skills/chenyu-yunying/assets/晨玙Amazon运营交付大母版.xlsx
+++ b/plugins/chenyu-yunying/skills/chenyu-yunying/assets/晨玙Amazon运营交付大母版.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品内容" sheetId="1" r:id="R900496e5b11f4772"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="作图要求" sheetId="2" r:id="R4a23fac1ccf54866"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DE Listing" sheetId="3" r:id="Rc44c7330780b4c83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR Listing" sheetId="4" r:id="Rb4e4aadddadc4d4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IT Listing" sheetId="5" r:id="R283c0dada03a4a08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ES Listing" sheetId="6" r:id="R3739771fb8194e96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品内容" sheetId="1" r:id="R0c3cb2e66f9c46f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="作图要求" sheetId="2" r:id="R076e57cebb7742b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DE Listing" sheetId="3" r:id="Rb24c56ba587241e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR Listing" sheetId="4" r:id="R4664c44c023f4bd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IT Listing" sheetId="5" r:id="R46fd4401d9444b9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ES Listing" sheetId="6" r:id="R8b30d26114d3418b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -241,7 +241,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd6a5d4bfd5a04bc5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2fd351239a234ce6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -273,7 +273,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R65a3a70257204a2e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4a1163c6dcad4e1b"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -300,7 +300,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R252542e411b24d16"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rcd7b8ae2b9ba485a"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -327,7 +327,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rca79bbecae334e76"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re34e09f29f2e4161"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -354,7 +354,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5b9cf932c2fc40e7"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4577067c41044c41"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -381,7 +381,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7d494548572d435b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rdbcaba0937eb44e5"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -408,7 +408,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb6f0141f50e5431e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra3bbc5381ab94cab"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -435,7 +435,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R32e79b8c758b4207"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R66cd9566fd40454a"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -462,7 +462,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc111b3108427483d"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R43c5033a021f4b54"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -489,7 +489,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R416ab74d4e9741cb"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R20995122cf3c4d93"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -516,7 +516,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb1d26941d7c84819"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rcbf707e94b0146bb"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -543,7 +543,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rce57643852bf4bda"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd82b1e6639554754"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -570,7 +570,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re36d55373c78428b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R17c2290143274188"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -597,7 +597,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc06e3b7ef77740b5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R292dec251bbb449a"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -624,7 +624,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rca1d19c73baa4026"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re8128ece84a34af6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -651,7 +651,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc35269f3986446b6"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2c9f3c8d553b468c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -678,7 +678,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R648fcbb642324313"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7d6d89993aa941f2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -705,7 +705,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Reedeca03a19a40c2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc72d09dd777f443d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -732,7 +732,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf317ebfba8df4467"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9f2e1d4ed0d14b6e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -759,7 +759,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R16327be6392941e8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R414cd28eb0ba4653"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1087,7 +1087,9 @@
         <x:v>变体1：圣诞小精灵-4个</x:v>
       </x:c>
       <x:c r="B2" s="8" t="str"/>
-      <x:c r="C2" s="8" t="str"/>
+      <x:c r="C2" s="8" t="str">
+        <x:v>同款竞品参考：单个总高约10.9 cm、最宽约5.0 cm（4.3 × 1.96 in）</x:v>
+      </x:c>
       <x:c r="D2" s="8" t="str"/>
       <x:c r="E2" s="8" t="str">
         <x:v>4个/套：红色×1、蓝色×1、绿色×1、粉色×1。开发表记录整套约200g；产品确认表记录单个约50g。</x:v>
@@ -1098,9 +1100,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re972525e629f4046"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R391688b069e84871"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d2e4d6cd7d94de3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a9c5793a2744bcc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1203,15 +1205,15 @@
       <x:c r="E4" s="20" t="str"/>
       <x:c r="F4" s="20" t="str"/>
       <x:c r="G4" s="29" t="str">
-        <x:v>参考图片1用于确定尺寸箭头方向、测量起止点和数值位置。
-参考图片2用于参考另一卖家的主尺寸、辅助尺寸和套装缩略图层级；不采用其尺寸与件数。
+        <x:v>参考图片1用于确定尺寸箭头方向、测量起止点和数值位置，并提供同款尺寸依据。
+参考图片2用于参考另一卖家的主尺寸、辅助尺寸和套装缩略图层级；不采用其件数。
 图片类型：尺寸图；成品数量：1张。
-画面目的：说明单个小精灵的真实尺寸，帮助买家判断摆放比例。
-制作前必补：实测单个产品从帽顶绒球最高点到鞋底的总高，以及身体/领口最宽处；用实测厘米换算英寸（1 in = 2.54 cm，英寸保留两位小数）。竞品图上的4.3 in和1.96 in只参考箭头版式，严禁直接采用。
-构图：选红色小精灵完整正面站立，中心测量区保持干净；竖向箭头标总高，横向箭头标最宽处；角落可放其余三色小缩略图或克制的松枝角饰，但不得遮挡箭头。
-上图文字：仅保留实测数值与单位，例如“__ cm / __ in”，不加说明性标题。
-禁止元素：估算尺寸、引用竞品尺寸、把帽高/身体宽误写成总高/总宽、夸大比例。
-验收：测量起止点明确；数值与实测记录一致；四款结构相同才允许共用同一组尺寸。
+画面目的：说明单个小精灵的总高和最宽处，帮助买家判断摆放比例。
+尺寸依据：开发资料未给出完整尺寸；已确认同款竞品标注总高4.3 in（约10.9 cm）、最宽1.96 in（约5.0 cm），本图可直接按该数值制作，无需等待自有实测。若后续实物测量与参考值不同，再以实测值更新。
+构图：选红色小精灵完整正面站立，中心测量区保持干净；竖向箭头从帽顶绒球最高点标到鞋底，标注10.9 cm / 4.3 in；横向箭头标身体或领口最宽处，标注5.0 cm / 1.96 in。角落可放其余三色小缩略图或克制的松枝角饰，但不得遮挡箭头。
+上图文字：仅保留“10.9 cm / 4.3 in”和“5.0 cm / 1.96 in”，不加说明性标题。
+禁止元素：混用非同款竞品尺寸、改变测量部位、把帽高或局部宽度误写成总高或总宽、夸大产品比例。
+验收：测量起止点明确；厘米与英寸换算正确；数值与已确认同款来源一致；四款结构相同，可共用同一组尺寸。
 输出：1:1，1254×1254 px。</x:v>
       </x:c>
     </x:row>
@@ -1314,9 +1316,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01a494c2cbf14647"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R464c44aa23034e53"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R834f0ce304b047f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b7b4ba27b294732"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1350,13 +1352,13 @@
         <x:v>Item Name</x:v>
       </x:c>
       <x:c r="B2" s="40" t="str">
-        <x:v>4 Mini Weihnachtselfen, Elfenpuppen und Wichtelfiguren für Advent</x:v>
+        <x:v>4 Mini Weihnachtselfen, Elfenpuppen und Wichtelfiguren für Adventsdeko</x:v>
       </x:c>
       <x:c r="C2" s="40" t="str">
-        <x:v>4个迷你圣诞小精灵，精灵玩偶和圣诞摆件，适用于降临节装饰。</x:v>
+        <x:v>4个迷你圣诞小精灵，精灵玩偶和小精灵摆件，适用于降临节装饰。</x:v>
       </x:c>
       <x:c r="D2" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP、B0CPJ65B1V 标题；开发文档 D3</x:v>
+        <x:v>开发文档 D3；参考 B0CLJ8J4RP、B0CPJ65B1V 标题</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="71.25" customHeight="1">
@@ -1364,13 +1366,13 @@
         <x:v>Item Highlights</x:v>
       </x:c>
       <x:c r="B3" s="40" t="str">
-        <x:v>4 Mini-Elfen in Rot, Blau, Grün und Rosa, ca. 10,9 cm, biegsam für Baum, Tisch, Regal und Adventsdeko</x:v>
+        <x:v>4 Mini-Elfen in Rot, Blau, Grün und Rosa, ca. 10.9 cm, biegsam für Baum, Tisch, Regal, Kaminsims, Fenster und Adventsdeko</x:v>
       </x:c>
       <x:c r="C3" s="40" t="str">
-        <x:v>红、蓝、绿、粉四色迷你圣诞小精灵4件套，单个约10.9 cm，手脚可弯折摆姿，可用于圣诞树、桌面、置物架和降临节布置。</x:v>
+        <x:v>红、蓝、绿、粉四色迷你圣诞小精灵4件套，单个约高10.9 cm，手脚可弯折摆姿，可用于圣诞树、桌面、置物架、壁炉架、窗台和降临节布置。</x:v>
       </x:c>
       <x:c r="D3" s="40" t="str">
-        <x:v>开发文档 D3、C3/F3；参考 B0CLJ8J4RP、B0CPJ65B1V</x:v>
+        <x:v>开发文档 D3、C3/F3；同款确认 I2/K2；参考 B0CLJ8J4RP、B0CPJ65B1V</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="165" customHeight="1">
@@ -1378,13 +1380,13 @@
         <x:v>五点 1</x:v>
       </x:c>
       <x:c r="B4" s="40" t="str">
-        <x:v>📦【4er-Set in vier Farben】Das Set enthält vier Mini-Elfen: je eine Figur in Rot, Blau, Grün und Rosa. Die festgelegte Farbmischung erleichtert ein abgestimmtes Arrangement, ohne zusätzliche Figuren oder Requisiten im Lieferumfang. Jede Farbe ist genau einmal enthalten, sodass der Lieferumfang sofort erkennbar bleibt und die vier Figuren gemeinsam oder verteilt dekoriert werden können.</x:v>
+        <x:v>📦【4er-Set in Rot, Blau, Grün und Rosa】Das Set enthält vier Mini-Weihnachtselfen, jeweils eine Figur in Rot, Blau, Grün und Rosa. Bei jeder Figur haben die spitze Mütze und der Anzug dieselbe Hauptfarbe, ergänzt durch einen weißen Mützenrand, einen weißen Blütenkragen und rote Schuhe.</x:v>
       </x:c>
       <x:c r="C4" s="40" t="str">
-        <x:v>📦【四色4件套】包装内含4个迷你圣诞小精灵，红、蓝、绿、粉各1个。固定的四色组合便于形成协调陈列，也能让买家清楚区分实际包装内容与场景道具。每种颜色仅包含1个，四个产品既可以成组摆放，也可以分别布置在不同位置。</x:v>
+        <x:v>📦【红蓝绿粉四色套装】套装包含4个迷你圣诞小精灵，红色、蓝色、绿色和粉色各1个。每个小精灵的尖顶帽与连体服采用相同主色，搭配白色帽檐、白色花瓣领和红色鞋子。</x:v>
       </x:c>
       <x:c r="D4" s="40" t="str">
-        <x:v>开发文档 D3；参考 B0CPJ65B1V 第2点</x:v>
+        <x:v>开发表四色/件数；自有图片帽子和服装颜色</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="165" customHeight="1">
@@ -1392,13 +1394,13 @@
         <x:v>五点 2</x:v>
       </x:c>
       <x:c r="B5" s="40" t="str">
-        <x:v>🧩【Biegbare Figuren für wechselnde Posen】Jede Figur ist etwa 10,9 cm hoch; Arme und Beine lassen sich biegen, sodass die kleinen Wichtel sitzen, stehen oder anders posieren können. So passt jede Elfenpuppe an verschiedene Dekoflächen. Die wiederkehrenden Details sorgen für ein einheitliches Gesamtbild, während Rot, Blau, Grün und Rosa im Set klar unterscheidbar bleiben.</x:v>
+        <x:v>🧩【Biegsame Arme und Beine】Die Arme und Beine der Elfen lassen sich für sitzende, stehende oder winkende Haltungen biegen. Für eine Sitzhaltung werden die Beine nach vorn gebeugt; die Arme können nach oben oder zur Seite zeigen, etwa beim Nachspielen einer Weihnachtsgeschichte mit den Elfen.</x:v>
       </x:c>
       <x:c r="C5" s="40" t="str">
-        <x:v>🧩【可弯折造型】每个小精灵约高10.9 cm，手臂和腿部可弯折，可根据展示需要调整为坐姿、站姿或其他姿态。不同姿势便于适配桌面、置物架和节日布景；四款保持相同造型细节，仅以红、蓝、绿、粉颜色进行区分。</x:v>
+        <x:v>🧩【手臂与双腿可弯折】小精灵的手臂和双腿可以弯折，可调整为坐姿、站姿或抬手姿势。双腿向前弯曲可呈现坐姿，双臂可朝上或朝向身体两侧调整，用于圣诞小精灵故事中的角色动作。</x:v>
       </x:c>
       <x:c r="D5" s="40" t="str">
-        <x:v>同款确认 I2/K2；参考 B0CLJ8J4RP 第1点、B0CPJ65B1V 第3点</x:v>
+        <x:v>同款 B0CLJ8J4RP 第1、4点；四肢可弯折</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="165" customHeight="1">
@@ -1406,13 +1408,13 @@
         <x:v>五点 3</x:v>
       </x:c>
       <x:c r="B6" s="40" t="str">
-        <x:v>🎄【Vielseitige Weihnachtsbaumdeko】Die Figuren eignen sich als Akzent am Weihnachtsbaum, auf dem Kaminsims, im Regal oder in einer festlichen Tischszene. Die vier Farben lassen sich einzeln verteilen oder als Gruppe arrangieren. So entsteht wahlweise ein gemeinsamer Blickfang oder mehrere kleine Weihnachtsakzente in unterschiedlichen Bereichen des Raums.</x:v>
+        <x:v>✨【Spitzmütze, Bommel und Lächeln】Jeder Elf besitzt große Augen, ein lächelndes Gesicht sowie hautfarbene Hände und eine hautfarbene Gesichtspartie. Die spitze Mütze trägt einen weißen Rand und Bommel; ein weißer blütenförmiger Kragen umgibt den Hals, während der Anzug Rumpf und Beine bedeckt und in roten Schuhen endet.</x:v>
       </x:c>
       <x:c r="C6" s="40" t="str">
-        <x:v>🎄【多场景圣诞装饰】可将小精灵布置在圣诞树旁、壁炉架、书架、玄关柜或节日餐桌上。四种颜色既能集中形成完整视觉焦点，也能分散到房间不同区域，作为多个小型圣诞点缀，同时保持整套产品的统一感。</x:v>
+        <x:v>✨【尖帽绒球与笑脸造型】小精灵带有大眼睛、微笑表情和肤色面部及双手，尖顶帽配有白色帽檐和帽顶绒球。白色花瓣形领口围绕颈部，衣服覆盖躯干及双腿，脚部为红色鞋子造型。</x:v>
       </x:c>
       <x:c r="D6" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP 第1点和第5点</x:v>
+        <x:v>自有图片面部、帽子、领口、手部和鞋子</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="165" customHeight="1">
@@ -1420,13 +1422,13 @@
         <x:v>五点 4</x:v>
       </x:c>
       <x:c r="B7" s="40" t="str">
-        <x:v>🎁【Kleines Adventsgeschenk】Die Mini-Elfen können als Strumpffüller, kleine Überraschung, Party-Mitgebsel oder dekorativer Geschenkanhänger verwendet werden. Jede Figur lässt sich einzeln verschenken oder im 4er-Set überreichen. Die vier einzelnen Figuren lassen sich außerdem auf mehrere Geschenkverpackungen, Adventsplätze oder Tischdekorationen verteilen.</x:v>
+        <x:v>📏【Miniaturgröße von etwa 10,9 cm】Jede Elfenfigur misst von der Mützenspitze bis zur Schuhsohle etwa 10,9 cm und ist an der breitesten Stelle etwa 5 cm breit. Das Miniaturformat eignet sich als Weihnachtsdekoration auf Kaminsims, Fensterbank, Bücherregal und Tisch sowie neben dem Weihnachtsbaum und in Adventsdekorationen.</x:v>
       </x:c>
       <x:c r="C7" s="40" t="str">
-        <x:v>🎁【降临节小礼物】迷你小精灵可作为圣诞袜填充小礼物、派对伴手礼、礼品包装点缀或节日小惊喜。4个产品可以整套赠送，也可以分别搭配多个礼盒、降临节布置或桌面装饰，便于根据场景灵活安排。</x:v>
+        <x:v>📏【约10.9厘米迷你尺寸】每个小精灵从帽顶到鞋底总高约10.9 cm，最宽处约5 cm。迷你尺寸适用于壁炉架、窗台、书架和桌面的圣诞摆件，也可用于圣诞树旁及降临节装饰。</x:v>
       </x:c>
       <x:c r="D7" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP 第2、3、5点；B0CPJ65B1V 第4点</x:v>
+        <x:v>同款 B0CLJ8J4RP 尺寸图及第1点</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="165" customHeight="1">
@@ -1434,27 +1436,27 @@
         <x:v>五点 5</x:v>
       </x:c>
       <x:c r="B8" s="40" t="str">
-        <x:v>✨【Zusammengehöriger Elf-Look】Spitze Mützen, weiße Kragen, freundliche Gesichter und rote Schuhe geben allen vier Figuren einen einheitlichen Stil. Das kompakte Format macht sie für kleine saisonale Dekoflächen geeignet. Alle sichtbaren Merkmale bleiben über die vier Farben hinweg gleich, sodass das Set als zusammengehörige Gruppe erkennbar ist.</x:v>
+        <x:v>🎁【Strumpffüller und Party-Mitgebsel】Die Mini-Elfen eignen sich als kleine Geschenke im Weihnachtsstrumpf, als Mitgebsel bei Weihnachtsfeiern oder als Figur auf einer Geschenkbox. Mit ihren Elfenanzügen sind sie kleine Weihnachtsgeschenke für Familienmitglieder und für Liebhaber gesammelter Miniaturfiguren zur Weihnachtszeit.</x:v>
       </x:c>
       <x:c r="C8" s="40" t="str">
-        <x:v>✨【统一精灵造型】尖顶帽、白色帽檐与绒球、白色花瓣形领口、笑脸和红色鞋子，让四个小精灵形成一致的节日造型。红、蓝、绿、粉四款沿用相同视觉元素，即使分开摆放也能保持整套产品的协调识别度。</x:v>
+        <x:v>🎁【圣诞袜礼物与派对赠礼】迷你小精灵可用作圣诞袜填充礼物、圣诞派对伴手礼及礼盒上的装饰。精灵服装和人物造型适合作为家人之间的圣诞小礼物，也适合喜欢收集迷你节日人物摆件的人。</x:v>
       </x:c>
       <x:c r="D8" s="40" t="str">
-        <x:v>开发文档 C3/F3；参考 B0CLJ8J4RP 图册02</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="285" customHeight="1">
+        <x:v>同款 B0CLJ8J4RP 第2、3、5点</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="390" customHeight="1">
       <x:c r="A9" s="39" t="str">
         <x:v>HTML 详情</x:v>
       </x:c>
       <x:c r="B9" s="40" t="str">
-        <x:v>&lt;p&gt;Vier kleine Weihnachtselfen in Rot, Blau, Grün und Rosa bringen einen abgestimmten Farbakzent in Advents- und Weihnachtsarrangements. Die Figuren sind etwa 10,9 cm hoch und können dank biegsamer Arme und Beine sitzend, stehend oder in einer individuellen Pose präsentiert werden.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Eigenschaften:&lt;/b&gt;&lt;br&gt;1. Vier Farben: Je eine Figur in Rot, Blau, Grün und Rosa.&lt;br&gt;2. Flexible Präsentation: Die Gliedmaßen lassen sich für unterschiedliche Posen biegen.&lt;br&gt;3. Festliche Gestaltung: Spitze Mützen, weiße Kragen, freundliche Gesichter und rote Schuhe.&lt;br&gt;4. Vielseitig kombinierbar: Für Baum, Regal, Kaminsims, Tischszene oder Geschenkdekoration.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Produktdetails:&lt;/b&gt;&lt;br&gt;Variante: 4er-Set&lt;br&gt;Höhe: ca. 10,9 cm je Figur&lt;br&gt;Farben: Rot, Blau, Grün und Rosa&lt;/p&gt;&lt;p&gt;&lt;b&gt;Lieferumfang:&lt;/b&gt;&lt;br&gt;4 × Mini-Weihnachtself&lt;/p&gt;</x:v>
+        <x:v>&lt;p&gt;Dieses Set enthält vier Mini-Weihnachtselfen in Rot, Blau, Grün und Rosa, jeweils eine Figur pro Farbe. Jede Figur ist etwa 10,9 cm hoch und 5 cm breit und besitzt biegsame Arme und Beine für Weihnachtsdekorationen, Figurengeschichten und kleine Geschenke.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Eigenschaften:&lt;/b&gt;&lt;br&gt;1. Vier Anzugfarben: Die vier Elfen tragen rote, blaue, grüne und rosa Anzüge mit jeweils farblich passender Spitzmütze. Mützenrand, Bommel und blütenförmiger Kragen sind weiß, die Schuhe sind rot.&lt;br&gt;2. Biegsame Gliedmaßen: Die Arme lassen sich nach oben oder seitlich ausrichten, die Beine für eine Sitzhaltung beugen. Auch stehende Haltungen sind möglich, etwa für Elfengeschichten und Figurenspiele in der Weihnachtszeit.&lt;br&gt;3. Maße und Figurendetails: Von der Mützenspitze bis zur Schuhsohle beträgt die Höhe etwa 10,9 cm, die Breite an der breitesten Stelle etwa 5 cm. Große Augen, ein lächelndes Gesicht, hautfarbene Hände, weißer Kragen und rote Schuhe gehören zu jeder Figur für Kaminsims, Regal oder Fensterbank.&lt;br&gt;4. Dekoration und kleine Geschenke: Die Figuren eignen sich für Weihnachtsdekorationen neben dem Baum und auf dem Tisch sowie als Strumpffüller oder Figur auf Geschenkboxen. Sie können als Weihnachtsmitgebsel an Familienmitglieder oder Sammler kleiner saisonaler Figuren verschenkt werden.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Produktdetails:&lt;/b&gt;&lt;br&gt;Anzahl: 4 Figuren&lt;br&gt;Farben: je 1 × Rot, Blau, Grün und Rosa&lt;br&gt;Gesamthöhe je Figur: etwa 10,9 cm&lt;br&gt;Größte Breite je Figur: etwa 5 cm&lt;br&gt;Ausführung: biegsame Arme und Beine&lt;/p&gt;&lt;p&gt;&lt;b&gt;Lieferumfang:&lt;/b&gt;&lt;br&gt;4 × Mini-Weihnachtself, je 1 × Rot, Blau, Grün und Rosa&lt;/p&gt;</x:v>
       </x:c>
       <x:c r="C9" s="40" t="str">
-        <x:v>&lt;p&gt;红、蓝、绿、粉四色圣诞小精灵各1个，可为降临节和圣诞节陈列增加协调的节日色彩。单个约高10.9 cm，手臂和腿部可弯折，可按展示需要调整坐姿、站姿或其他姿态。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品特点：&lt;/b&gt;&lt;br&gt;1. 四色组合：红、蓝、绿、粉各1个，共4个。&lt;br&gt;2. 灵活摆放：可调整手脚姿态，适合不同陈列方式。&lt;br&gt;3. 节日造型：尖顶帽、白色领口、笑脸和红色鞋子。&lt;br&gt;4. 多种场景：适用于圣诞树、书架、壁炉架、桌面和礼品包装。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品参数：&lt;/b&gt;&lt;br&gt;规格：4件套&lt;br&gt;高度：单个约10.9 cm&lt;br&gt;颜色：红、蓝、绿、粉&lt;/p&gt;&lt;p&gt;&lt;b&gt;包装内容：&lt;/b&gt;&lt;br&gt;4 × 迷你圣诞小精灵&lt;/p&gt;</x:v>
+        <x:v>&lt;p&gt;这套迷你圣诞小精灵包含红、蓝、绿、粉四种颜色，各1个。单个约高10.9 cm、最宽约5 cm，手臂和双腿可弯折，适用于圣诞家居装饰、节日人物故事及小礼物。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品特点:&lt;/b&gt;&lt;br&gt;1. 四色服装: 四个小精灵分别穿红、蓝、绿、粉色连体服，尖顶帽与服装主色相配。帽檐、帽顶绒球和花瓣形领口为白色，鞋子为红色。&lt;br&gt;2. 可弯折四肢: 手臂可调整为抬起或位于身体两侧的姿势，双腿可弯曲呈坐姿。也可调整为站姿，用于圣诞小精灵故事和人物游戏。&lt;br&gt;3. 尺寸与外观: 从帽顶到鞋底总高约10.9 cm，最宽处约5 cm。大眼笑脸、肤色双手、白色领口和红色鞋子是每个小精灵的造型细节，可放在壁炉架、书架或窗台。&lt;br&gt;4. 节日装饰与赠礼: 可用作圣诞树旁和桌面的节日人物摆件，也可放入圣诞袜或作为礼盒装饰。适合作为圣诞派对小礼物，赠给家人或迷你节日人物收藏爱好者。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品参数:&lt;/b&gt;&lt;br&gt;数量：4个&lt;br&gt;颜色：红、蓝、绿、粉各1个&lt;br&gt;单个总高：约10.9 cm&lt;br&gt;单个最宽处：约5 cm&lt;br&gt;结构：手臂和双腿可弯折&lt;/p&gt;&lt;p&gt;&lt;b&gt;包装内容:&lt;/b&gt;&lt;br&gt;4 × 迷你圣诞小精灵，红、蓝、绿、粉各1个&lt;/p&gt;</x:v>
       </x:c>
       <x:c r="D9" s="40" t="str">
-        <x:v>开发文档 D3、C3/F3；参考 B0CLJ8J4RP 第1-5点</x:v>
+        <x:v>自有颜色、数量及图片；同款 B0CLJ8J4RP 第1–5点及尺寸图</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="75" customHeight="1">
@@ -1462,19 +1464,19 @@
         <x:v>Search Terms</x:v>
       </x:c>
       <x:c r="B10" s="40" t="str">
-        <x:v>koboldpüppchen festtagsornament nikolausbeigabe adventskalenderfüllung winterarrangement schaufensterakzent</x:v>
+        <x:v>wichtelmännchen dekofigur aufsteller kobold schaufensterschmuck winterfigur nikolausbeigabe adventskalenderfüllung festtagsornament tischfigur weihnachtszwerg zwergpuppe tomte gnom winterdeko kaminfigur</x:v>
       </x:c>
       <x:c r="C10" s="40" t="str">
-        <x:v>小妖精玩偶 节日摆件 圣诞小礼物 降临节日历填充物 冬季布置 橱窗点缀</x:v>
+        <x:v>小精灵 装饰摆件 立式摆件 小妖精 橱窗装饰 冬季人偶 圣尼古拉节小礼物 降临节日历填充物 节日饰品 桌面人偶 圣诞小矮人 小矮人玩偶 北欧地精 地精 冬季装饰 壁炉人偶</x:v>
       </x:c>
       <x:c r="D10" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP、B0CPJ65B1V 标题及五点/关键词提取</x:v>
+        <x:v>既有同款关键词候选；Amazon DE“weihnachtspuppe wichtel kobold”前20个结果复核；参考 B0CLJ8J4RP、B0CPJ65B1V 标题</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf2e0c545a4c48d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e5860d4275944fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1508,13 +1510,13 @@
         <x:v>Item Name</x:v>
       </x:c>
       <x:c r="B2" s="40" t="str">
-        <x:v>Lot de 4 mini lutins, poupées elfes et figurines de Noël pour l’Avent</x:v>
+        <x:v>Lot de 4 mini lutins de Noël, poupées elfes et figurines déco pour l’Avent</x:v>
       </x:c>
       <x:c r="C2" s="40" t="str">
-        <x:v>4个迷你圣诞小精灵，精灵玩偶和圣诞摆件，适用于降临节装饰。</x:v>
+        <x:v>4个迷你圣诞小精灵，精灵玩偶及装饰摆件，适用于降临节布置。</x:v>
       </x:c>
       <x:c r="D2" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP、B0CPJ65B1V 标题；开发文档 D3</x:v>
+        <x:v>开发文档 D3；参考 B0CLJ8J4RP、B0CPJ65B1V 标题</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="71.25" customHeight="1">
@@ -1522,13 +1524,13 @@
         <x:v>Item Highlights</x:v>
       </x:c>
       <x:c r="B3" s="40" t="str">
-        <x:v>4 mini lutins rouge, bleu, vert et rose, env. 10,9 cm, pliables pour sapin, table, étagère et décor de l’Avent</x:v>
+        <x:v>4 mini lutins rouge, bleu, vert et rose, env. 10.9 cm, pliables pour sapin, table, étagère, cheminée et décor de l’Avent</x:v>
       </x:c>
       <x:c r="C3" s="40" t="str">
-        <x:v>红、蓝、绿、粉四色迷你圣诞小精灵4件套，单个约10.9 cm，手脚可弯折摆姿，可用于圣诞树、桌面、置物架和降临节布置。</x:v>
+        <x:v>红、蓝、绿、粉四色迷你圣诞小精灵4件套，单个约高10.9 cm，手脚可弯折摆姿，可用于圣诞树、桌面、置物架、壁炉架和降临节布置。</x:v>
       </x:c>
       <x:c r="D3" s="40" t="str">
-        <x:v>开发文档 D3、C3/F3；参考 B0CLJ8J4RP、B0CPJ65B1V</x:v>
+        <x:v>开发文档 D3、C3/F3；同款确认 I2/K2；参考 B0CLJ8J4RP、B0CPJ65B1V</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="165" customHeight="1">
@@ -1536,13 +1538,13 @@
         <x:v>五点 1</x:v>
       </x:c>
       <x:c r="B4" s="40" t="str">
-        <x:v>📦【Lot de quatre couleurs】Le lot comprend quatre mini lutins, un rouge, un bleu, un vert et un rose. Cette composition définie permet de créer un ensemble coordonné sans confondre les accessoires de mise en scène avec le contenu du paquet. Chaque couleur est présente une seule fois, ce qui permet d’identifier immédiatement le contenu et de placer les quatre personnages ensemble ou séparément.</x:v>
+        <x:v>📦【Lot de 4 en rouge, bleu, vert et rose】Le lot comprend quatre mini lutins de Noël : un rouge, un bleu, un vert et un rose. Le bonnet pointu et la combinaison de chaque personnage ont la même couleur principale, avec un bord de bonnet blanc, un col blanc en pétales et des chaussures rouges.</x:v>
       </x:c>
       <x:c r="C4" s="40" t="str">
-        <x:v>📦【四色4件套】包装内含4个迷你圣诞小精灵，红、蓝、绿、粉各1个。固定的四色组合便于形成协调陈列，也能让买家清楚区分实际包装内容与场景道具。每种颜色仅包含1个，四个产品既可以成组摆放，也可以分别布置在不同位置。</x:v>
+        <x:v>📦【红蓝绿粉四色套装】套装包含4个迷你圣诞小精灵，红色、蓝色、绿色和粉色各1个。每个小精灵的尖顶帽与连体服采用相同主色，搭配白色帽檐、白色花瓣领和红色鞋子。</x:v>
       </x:c>
       <x:c r="D4" s="40" t="str">
-        <x:v>开发文档 D3；参考 B0CPJ65B1V 第2点</x:v>
+        <x:v>开发表四色/件数；自有图片帽子和服装颜色</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="165" customHeight="1">
@@ -1550,13 +1552,13 @@
         <x:v>五点 2</x:v>
       </x:c>
       <x:c r="B5" s="40" t="str">
-        <x:v>🧩【Figurines articulées】Chaque lutin mesure environ 10,9 cm et ses bras et jambes se plient pour adopter une position assise, debout ou inclinée. Les poupées elfes s’adaptent ainsi à différentes surfaces décoratives. Les détails répétés créent un ensemble visuel cohérent, tandis que le rouge, le bleu, le vert et le rose restent faciles à distinguer.</x:v>
+        <x:v>🧩【Bras et jambes pliables】Les bras et les jambes des lutins se plient pour obtenir des positions assises, debout ou avec les bras levés. Les jambes se replient vers l’avant pour une posture assise, tandis que les bras peuvent être orientés vers le haut ou sur les côtés pour jouer les personnages des histoires de Noël.</x:v>
       </x:c>
       <x:c r="C5" s="40" t="str">
-        <x:v>🧩【可弯折造型】每个小精灵约高10.9 cm，手臂和腿部可弯折，可根据展示需要调整为坐姿、站姿或其他姿态。不同姿势便于适配桌面、置物架和节日布景；四款保持相同造型细节，仅以红、蓝、绿、粉颜色进行区分。</x:v>
+        <x:v>🧩【手臂与双腿可弯折】小精灵的手臂和双腿可以弯折，可调整为坐姿、站姿或抬手姿势。双腿向前弯曲可呈现坐姿，双臂可朝上或朝向身体两侧调整，用于圣诞小精灵故事中的角色动作。</x:v>
       </x:c>
       <x:c r="D5" s="40" t="str">
-        <x:v>同款确认 I2/K2；参考 B0CLJ8J4RP 第1点、B0CPJ65B1V 第3点</x:v>
+        <x:v>同款 B0CLJ8J4RP 第1、4点；四肢可弯折</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="165" customHeight="1">
@@ -1564,13 +1566,13 @@
         <x:v>五点 3</x:v>
       </x:c>
       <x:c r="B6" s="40" t="str">
-        <x:v>🎄【Décoration de sapin polyvalente】Disposez les lutins près du sapin, sur une étagère, un manteau de cheminée ou au centre d’une table de fête. Les quatre couleurs peuvent être réparties dans la pièce ou réunies en petit groupe. Vous pouvez ainsi créer un point focal commun ou répartir plusieurs petits accents de Noël dans différentes zones de la pièce.</x:v>
+        <x:v>✨【Bonnet à pompon et visage souriant】Chaque lutin possède de grands yeux, un visage souriant, ainsi que des mains et un visage couleur chair. Le bonnet pointu est bordé de blanc et terminé par un pompon blanc ; un col blanc en pétales entoure le cou, la combinaison couvre le buste et les jambes et se termine par des chaussures rouges.</x:v>
       </x:c>
       <x:c r="C6" s="40" t="str">
-        <x:v>🎄【多场景圣诞装饰】可将小精灵布置在圣诞树旁、壁炉架、书架、玄关柜或节日餐桌上。四种颜色既能集中形成完整视觉焦点，也能分散到房间不同区域，作为多个小型圣诞点缀，同时保持整套产品的统一感。</x:v>
+        <x:v>✨【尖帽绒球与笑脸造型】小精灵带有大眼睛、微笑表情和肤色面部及双手，尖顶帽配有白色帽檐和帽顶绒球。白色花瓣形领口围绕颈部，衣服覆盖躯干及双腿，脚部为红色鞋子造型。</x:v>
       </x:c>
       <x:c r="D6" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP 第1点和第5点</x:v>
+        <x:v>自有图片面部、帽子、领口、手部和鞋子</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="165" customHeight="1">
@@ -1578,13 +1580,13 @@
         <x:v>五点 4</x:v>
       </x:c>
       <x:c r="B7" s="40" t="str">
-        <x:v>🎁【Petit cadeau de l’Avent】Chaque figurine peut servir de petite surprise, de cadeau d’invité, de garniture de chaussette ou d’ornement pour un paquet. Le lot peut être offert ensemble ou réparti entre plusieurs personnes. Les quatre figurines peuvent également être réparties sur plusieurs paquets, coins de l’Avent ou décorations de table selon la présentation souhaitée.</x:v>
+        <x:v>📏【Format miniature d’environ 10,9 cm】Chaque figurine mesure environ 10,9 cm du sommet du bonnet à la semelle des chaussures et environ 5 cm au point le plus large. Ce format miniature convient à une décoration de Noël sur une cheminée, un rebord de fenêtre, une bibliothèque ou une table, près du sapin ou dans un décor de l’Avent.</x:v>
       </x:c>
       <x:c r="C7" s="40" t="str">
-        <x:v>🎁【降临节小礼物】迷你小精灵可作为圣诞袜填充小礼物、派对伴手礼、礼品包装点缀或节日小惊喜。4个产品可以整套赠送，也可以分别搭配多个礼盒、降临节布置或桌面装饰，便于根据场景灵活安排。</x:v>
+        <x:v>📏【约10.9厘米迷你尺寸】每个小精灵从帽顶到鞋底总高约10.9 cm，最宽处约5 cm。迷你尺寸适用于壁炉架、窗台、书架和桌面的圣诞摆件，也可用于圣诞树旁及降临节装饰。</x:v>
       </x:c>
       <x:c r="D7" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP 第2、3、5点；B0CPJ65B1V 第4点</x:v>
+        <x:v>同款 B0CLJ8J4RP 尺寸图及第1点</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="165" customHeight="1">
@@ -1592,27 +1594,27 @@
         <x:v>五点 5</x:v>
       </x:c>
       <x:c r="B8" s="40" t="str">
-        <x:v>✨【Style elfe coordonné】Les bonnets pointus, les cols blancs, les visages souriants et les chaussures rouges donnent aux quatre personnages une apparence cohérente. Leur format compact convient aux petits espaces de décoration saisonnière. Les mêmes éléments visuels sont conservés sur les quatre couleurs afin que le lot reste immédiatement reconnaissable comme un ensemble coordonné.</x:v>
+        <x:v>🎁【Chaussettes et cadeaux d’invités】Les mini lutins peuvent garnir une chaussette de Noël, servir de cadeaux d’invités pour une fête de Noël ou décorer un paquet cadeau. Leurs tenues de lutins en font de petites attentions de Noël pour la famille et pour les amateurs de figurines miniatures de saison.</x:v>
       </x:c>
       <x:c r="C8" s="40" t="str">
-        <x:v>✨【统一精灵造型】尖顶帽、白色帽檐与绒球、白色花瓣形领口、笑脸和红色鞋子，让四个小精灵形成一致的节日造型。红、蓝、绿、粉四款沿用相同视觉元素，即使分开摆放也能保持整套产品的协调识别度。</x:v>
+        <x:v>🎁【圣诞袜礼物与派对赠礼】迷你小精灵可用作圣诞袜填充礼物、圣诞派对伴手礼及礼盒上的装饰。精灵服装和人物造型适合作为家人之间的圣诞小礼物，也适合喜欢收集迷你节日人物摆件的人。</x:v>
       </x:c>
       <x:c r="D8" s="40" t="str">
-        <x:v>开发文档 C3/F3；参考 B0CLJ8J4RP 图册02</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="285" customHeight="1">
+        <x:v>同款 B0CLJ8J4RP 第2、3、5点</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="390" customHeight="1">
       <x:c r="A9" s="39" t="str">
         <x:v>HTML 详情</x:v>
       </x:c>
       <x:c r="B9" s="40" t="str">
-        <x:v>&lt;p&gt;Ces quatre mini lutins de Noël, en rouge, bleu, vert et rose, ajoutent une touche coordonnée aux décors de l’Avent. Chaque figurine mesure environ 10,9 cm et possède des bras et des jambes pliables pour varier les positions.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Caractéristiques :&lt;/b&gt;&lt;br&gt;1. Quatre couleurs : un lutin rouge, un bleu, un vert et un rose.&lt;br&gt;2. Présentation modulable : position assise, debout ou inclinée.&lt;br&gt;3. Détails festifs : bonnet pointu, col blanc, visage souriant et chaussures rouges.&lt;br&gt;4. Utilisation variée : sapin, étagère, manteau de cheminée, table ou emballage cadeau.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Informations sur le produit :&lt;/b&gt;&lt;br&gt;Variante : lot de 4&lt;br&gt;Hauteur : environ 10,9 cm par figurine&lt;br&gt;Couleurs : rouge, bleu, vert et rose&lt;/p&gt;&lt;p&gt;&lt;b&gt;Contenu de l’emballage :&lt;/b&gt;&lt;br&gt;4 × mini lutin de Noël&lt;/p&gt;</x:v>
+        <x:v>&lt;p&gt;Ce lot contient quatre mini lutins de Noël, un rouge, un bleu, un vert et un rose. Chaque figurine mesure environ 10,9 cm de haut et 5 cm de large, avec des bras et des jambes pliables pour la décoration de Noël, les histoires de personnages et les petits cadeaux.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Caractéristiques:&lt;/b&gt;&lt;br&gt;1. Quatre couleurs de tenues: Les quatre lutins portent des combinaisons rouge, bleue, verte et rose avec un bonnet pointu assorti. Le bord du bonnet, le pompon et le col en pétales sont blancs, les chaussures sont rouges.&lt;br&gt;2. Membres pliables: Les bras peuvent être levés ou placés sur les côtés, et les jambes repliées pour une posture assise. Une position debout est également possible pour les histoires de lutins et les jeux de personnages à Noël.&lt;br&gt;3. Dimensions et détails: La hauteur du sommet du bonnet à la semelle est d’environ 10,9 cm, pour environ 5 cm au point le plus large. Grands yeux, sourire, mains couleur chair, col blanc et chaussures rouges composent chaque figurine à poser sur une cheminée, une étagère ou un rebord de fenêtre.&lt;br&gt;4. Décoration et petits cadeaux: Les personnages conviennent aux décors de Noël près du sapin ou sur une table, ainsi qu’aux chaussettes et aux paquets cadeaux. Ils peuvent être offerts lors d’une fête de Noël à des proches ou à des amateurs de petites figurines saisonnières.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Informations sur le produit:&lt;/b&gt;&lt;br&gt;Quantité : 4 figurines&lt;br&gt;Couleurs : 1 × rouge, bleu, vert et rose&lt;br&gt;Hauteur totale par figurine : environ 10,9 cm&lt;br&gt;Largeur maximale par figurine : environ 5 cm&lt;br&gt;Structure : bras et jambes pliables&lt;/p&gt;&lt;p&gt;&lt;b&gt;Contenu de l’emballage:&lt;/b&gt;&lt;br&gt;4 × mini lutin de Noël, un rouge, un bleu, un vert et un rose&lt;/p&gt;</x:v>
       </x:c>
       <x:c r="C9" s="40" t="str">
-        <x:v>&lt;p&gt;红、蓝、绿、粉四色圣诞小精灵各1个，可为降临节和圣诞节陈列增加协调的节日色彩。单个约高10.9 cm，手臂和腿部可弯折，可按展示需要调整坐姿、站姿或其他姿态。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品特点：&lt;/b&gt;&lt;br&gt;1. 四色组合：红、蓝、绿、粉各1个，共4个。&lt;br&gt;2. 灵活摆放：可调整手脚姿态，适合不同陈列方式。&lt;br&gt;3. 节日造型：尖顶帽、白色领口、笑脸和红色鞋子。&lt;br&gt;4. 多种场景：适用于圣诞树、书架、壁炉架、桌面和礼品包装。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品参数：&lt;/b&gt;&lt;br&gt;规格：4件套&lt;br&gt;高度：单个约10.9 cm&lt;br&gt;颜色：红、蓝、绿、粉&lt;/p&gt;&lt;p&gt;&lt;b&gt;包装内容：&lt;/b&gt;&lt;br&gt;4 × 迷你圣诞小精灵&lt;/p&gt;</x:v>
+        <x:v>&lt;p&gt;这套迷你圣诞小精灵包含红、蓝、绿、粉四种颜色，各1个。单个约高10.9 cm、最宽约5 cm，手臂和双腿可弯折，适用于圣诞家居装饰、节日人物故事及小礼物。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品特点:&lt;/b&gt;&lt;br&gt;1. 四色服装: 四个小精灵分别穿红、蓝、绿、粉色连体服，尖顶帽与服装主色相配。帽檐、帽顶绒球和花瓣形领口为白色，鞋子为红色。&lt;br&gt;2. 可弯折四肢: 手臂可调整为抬起或位于身体两侧的姿势，双腿可弯曲呈坐姿。也可调整为站姿，用于圣诞小精灵故事和人物游戏。&lt;br&gt;3. 尺寸与外观: 从帽顶到鞋底总高约10.9 cm，最宽处约5 cm。大眼笑脸、肤色双手、白色领口和红色鞋子是每个小精灵的造型细节，可放在壁炉架、书架或窗台。&lt;br&gt;4. 节日装饰与赠礼: 可用作圣诞树旁和桌面的节日人物摆件，也可放入圣诞袜或作为礼盒装饰。适合作为圣诞派对小礼物，赠给家人或迷你节日人物收藏爱好者。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品参数:&lt;/b&gt;&lt;br&gt;数量：4个&lt;br&gt;颜色：红、蓝、绿、粉各1个&lt;br&gt;单个总高：约10.9 cm&lt;br&gt;单个最宽处：约5 cm&lt;br&gt;结构：手臂和双腿可弯折&lt;/p&gt;&lt;p&gt;&lt;b&gt;包装内容:&lt;/b&gt;&lt;br&gt;4 × 迷你圣诞小精灵，红、蓝、绿、粉各1个&lt;/p&gt;</x:v>
       </x:c>
       <x:c r="D9" s="40" t="str">
-        <x:v>开发文档 D3、C3/F3；参考 B0CLJ8J4RP 第1-5点</x:v>
+        <x:v>自有颜色、数量及图片；同款 B0CLJ8J4RP 第1–5点及尺寸图</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="75" customHeight="1">
@@ -1620,19 +1622,19 @@
         <x:v>Search Terms</x:v>
       </x:c>
       <x:c r="B10" s="40" t="str">
-        <x:v>farfadets bibelots calendrier sachets invités vitrine hivernale</x:v>
+        <x:v>farfadets santons bibelots calendrier présentoir vitrine hivernale statuettes nains tomte gonk sujets farceurs bonshommes village</x:v>
       </x:c>
       <x:c r="C10" s="40" t="str">
-        <x:v>小精灵 装饰摆件 日历 礼袋填充物 冬季橱窗</x:v>
+        <x:v>小精灵 圣诞人物小雕像 装饰摆件 日历 陈列架 橱窗 冬季 小雕像 小矮人 北欧地精 地精 装饰人物 淘气精灵 小人偶 村庄</x:v>
       </x:c>
       <x:c r="D10" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP、B0CPJ65B1V 标题及五点/关键词提取</x:v>
+        <x:v>既有同款关键词候选及参考标题本地化；Amazon FR 本次页面访问受限，未声称当地搜索量</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R955ff4ff59cb4358"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1443facdec1a49e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1666,13 +1668,13 @@
         <x:v>Item Name</x:v>
       </x:c>
       <x:c r="B2" s="40" t="str">
-        <x:v>Set 4 mini elfi di Natale, bambole elfo e statuine per l’Avvento</x:v>
+        <x:v>Set 4 mini elfi di Natale, bambole elfo e statuine decorative per l’Avvento</x:v>
       </x:c>
       <x:c r="C2" s="40" t="str">
-        <x:v>4个迷你圣诞小精灵，精灵玩偶和圣诞摆件，适用于降临节装饰。</x:v>
+        <x:v>4个迷你圣诞小精灵，精灵玩偶和装饰摆件，适用于降临节布置。</x:v>
       </x:c>
       <x:c r="D2" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP、B0CPJ65B1V 标题；开发文档 D3</x:v>
+        <x:v>开发文档 D3；参考 B0CLJ8J4RP、B0CPJ65B1V 标题</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="71.25" customHeight="1">
@@ -1680,13 +1682,13 @@
         <x:v>Item Highlights</x:v>
       </x:c>
       <x:c r="B3" s="40" t="str">
-        <x:v>4 mini elfi rossi, blu, verdi e rosa, circa 10,9 cm, pieghevoli per albero, tavolo, mensola e decorazioni</x:v>
+        <x:v>4 mini elfi rossi, blu, verdi e rosa, circa 10.9 cm, pieghevoli per albero, tavolo, mensola, camino e decorazioni natalizie</x:v>
       </x:c>
       <x:c r="C3" s="40" t="str">
-        <x:v>红、蓝、绿、粉四色迷你圣诞小精灵4件套，单个约10.9 cm，手脚可弯折摆姿，可用于圣诞树、桌面、置物架和降临节布置。</x:v>
+        <x:v>红、蓝、绿、粉四色迷你圣诞小精灵4件套，单个约高10.9 cm，手脚可弯折摆姿，可用于圣诞树、桌面、置物架、壁炉架和圣诞布置。</x:v>
       </x:c>
       <x:c r="D3" s="40" t="str">
-        <x:v>开发文档 D3、C3/F3；参考 B0CLJ8J4RP、B0CPJ65B1V</x:v>
+        <x:v>开发文档 D3、C3/F3；同款确认 I2/K2；参考 B0CLJ8J4RP、B0CPJ65B1V</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="165" customHeight="1">
@@ -1694,13 +1696,13 @@
         <x:v>五点 1</x:v>
       </x:c>
       <x:c r="B4" s="40" t="str">
-        <x:v>📦【Set da quattro colori】La confezione contiene quattro mini elfi: uno rosso, uno blu, uno verde e uno rosa. La combinazione già definita crea un insieme coordinato e distingue chiaramente le statuine dagli oggetti usati solo nella scena. Ogni colore è presente una sola volta, così il contenuto della confezione resta immediato e le quattro figure possono essere esposte insieme oppure separate.</x:v>
+        <x:v>📦【Set da 4 in rosso, blu, verde e rosa】Il set comprende quattro mini elfi di Natale: uno rosso, uno blu, uno verde e uno rosa. Il cappello a punta e la tuta di ogni personaggio hanno lo stesso colore principale, con bordo del cappello bianco, colletto bianco a petali e scarpe rosse.</x:v>
       </x:c>
       <x:c r="C4" s="40" t="str">
-        <x:v>📦【四色4件套】包装内含4个迷你圣诞小精灵，红、蓝、绿、粉各1个。固定的四色组合便于形成协调陈列，也能让买家清楚区分实际包装内容与场景道具。每种颜色仅包含1个，四个产品既可以成组摆放，也可以分别布置在不同位置。</x:v>
+        <x:v>📦【红蓝绿粉四色套装】套装包含4个迷你圣诞小精灵，红色、蓝色、绿色和粉色各1个。每个小精灵的尖顶帽与连体服采用相同主色，搭配白色帽檐、白色花瓣领和红色鞋子。</x:v>
       </x:c>
       <x:c r="D4" s="40" t="str">
-        <x:v>开发文档 D3；参考 B0CPJ65B1V 第2点</x:v>
+        <x:v>开发表四色/件数；自有图片帽子和服装颜色</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="165" customHeight="1">
@@ -1708,13 +1710,13 @@
         <x:v>五点 2</x:v>
       </x:c>
       <x:c r="B5" s="40" t="str">
-        <x:v>🧩【Figure snodabili】Ogni elfo è alto circa 10,9 cm e ha braccia e gambe pieghevoli per essere esposto seduto, in piedi o in altre pose. Le bambole elfo si adattano così a ripiani e composizioni diverse. I dettagli ripetuti creano un aspetto coordinato, mentre rosso, blu, verde e rosa restano chiaramente distinguibili all’interno del set.</x:v>
+        <x:v>🧩【Braccia e gambe pieghevoli】Le braccia e le gambe degli elfi si piegano per ottenere posizioni sedute, in piedi o con le braccia alzate. Le gambe si piegano in avanti per la posizione seduta, mentre le braccia possono essere rivolte verso l’alto o ai lati per interpretare i personaggi delle storie di Natale.</x:v>
       </x:c>
       <x:c r="C5" s="40" t="str">
-        <x:v>🧩【可弯折造型】每个小精灵约高10.9 cm，手臂和腿部可弯折，可根据展示需要调整为坐姿、站姿或其他姿态。不同姿势便于适配桌面、置物架和节日布景；四款保持相同造型细节，仅以红、蓝、绿、粉颜色进行区分。</x:v>
+        <x:v>🧩【手臂与双腿可弯折】小精灵的手臂和双腿可以弯折，可调整为坐姿、站姿或抬手姿势。双腿向前弯曲可呈现坐姿，双臂可朝上或朝向身体两侧调整，用于圣诞小精灵故事中的角色动作。</x:v>
       </x:c>
       <x:c r="D5" s="40" t="str">
-        <x:v>同款确认 I2/K2；参考 B0CLJ8J4RP 第1点、B0CPJ65B1V 第3点</x:v>
+        <x:v>同款 B0CLJ8J4RP 第1、4点；四肢可弯折</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="165" customHeight="1">
@@ -1722,13 +1724,13 @@
         <x:v>五点 3</x:v>
       </x:c>
       <x:c r="B6" s="40" t="str">
-        <x:v>🎄【Decorazione per albero versatile】Sistema gli elfi vicino all’albero, su una mensola, sul caminetto o al centro di una tavola festiva. I quattro colori possono essere distribuiti nello spazio oppure riuniti in un piccolo gruppo. In questo modo puoi creare un unico punto decorativo oppure distribuire piccoli accenti natalizi in diverse zone della stanza.</x:v>
+        <x:v>✨【Cappello con pompon e viso sorridente】Ogni elfo ha grandi occhi, un viso sorridente e mani e volto color carne. Il cappello a punta presenta bordo e pompon bianchi; un colletto bianco a petali circonda il collo, la tuta copre busto e gambe e termina con scarpe rosse.</x:v>
       </x:c>
       <x:c r="C6" s="40" t="str">
-        <x:v>🎄【多场景圣诞装饰】可将小精灵布置在圣诞树旁、壁炉架、书架、玄关柜或节日餐桌上。四种颜色既能集中形成完整视觉焦点，也能分散到房间不同区域，作为多个小型圣诞点缀，同时保持整套产品的统一感。</x:v>
+        <x:v>✨【尖帽绒球与笑脸造型】小精灵带有大眼睛、微笑表情和肤色面部及双手，尖顶帽配有白色帽檐和帽顶绒球。白色花瓣形领口围绕颈部，衣服覆盖躯干及双腿，脚部为红色鞋子造型。</x:v>
       </x:c>
       <x:c r="D6" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP 第1点和第5点</x:v>
+        <x:v>自有图片面部、帽子、领口、手部和鞋子</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="165" customHeight="1">
@@ -1736,13 +1738,13 @@
         <x:v>五点 4</x:v>
       </x:c>
       <x:c r="B7" s="40" t="str">
-        <x:v>🎁【Piccolo regalo dell’Avvento】Le statuine possono essere usate come sorpresa, pensierino per gli ospiti, riempitivo per calza o segnapacco decorativo. Puoi regalare l’intero set oppure dividere i quattro personaggi. Le quattro statuine possono anche essere suddivise tra più pacchi regalo, angoli dell’Avvento o composizioni da tavola in base all’allestimento.</x:v>
+        <x:v>📏【Formato mini da circa 10,9 cm】Ogni statuina misura circa 10,9 cm dalla punta del cappello alla suola delle scarpe e circa 5 cm nel punto più largo. Il formato mini è adatto alle decorazioni natalizie su camino, davanzale, libreria e tavolo, accanto all’albero o negli allestimenti dell’Avvento.</x:v>
       </x:c>
       <x:c r="C7" s="40" t="str">
-        <x:v>🎁【降临节小礼物】迷你小精灵可作为圣诞袜填充小礼物、派对伴手礼、礼品包装点缀或节日小惊喜。4个产品可以整套赠送，也可以分别搭配多个礼盒、降临节布置或桌面装饰，便于根据场景灵活安排。</x:v>
+        <x:v>📏【约10.9厘米迷你尺寸】每个小精灵从帽顶到鞋底总高约10.9 cm，最宽处约5 cm。迷你尺寸适用于壁炉架、窗台、书架和桌面的圣诞摆件，也可用于圣诞树旁及降临节装饰。</x:v>
       </x:c>
       <x:c r="D7" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP 第2、3、5点；B0CPJ65B1V 第4点</x:v>
+        <x:v>同款 B0CLJ8J4RP 尺寸图及第1点</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="165" customHeight="1">
@@ -1750,27 +1752,27 @@
         <x:v>五点 5</x:v>
       </x:c>
       <x:c r="B8" s="40" t="str">
-        <x:v>✨【Aspetto coordinato da elfo】Cappelli a punta, colletti bianchi, visi sorridenti e scarpe rosse danno ai quattro personaggi uno stile coerente. Il formato compatto è adatto anche a spazi decorativi stagionali ridotti. Gli stessi elementi visivi ricorrono in tutti e quattro i colori, rendendo il set riconoscibile come gruppo coordinato anche quando viene distribuito.</x:v>
+        <x:v>🎁【Regalini per calze e feste di Natale】I mini elfi possono riempire una calza natalizia, essere offerti agli invitati di una festa di Natale o decorare un pacco regalo. Le loro tute da elfo li rendono piccoli pensieri natalizi per i familiari e per chi colleziona personaggi in miniatura a tema festivo.</x:v>
       </x:c>
       <x:c r="C8" s="40" t="str">
-        <x:v>✨【统一精灵造型】尖顶帽、白色帽檐与绒球、白色花瓣形领口、笑脸和红色鞋子，让四个小精灵形成一致的节日造型。红、蓝、绿、粉四款沿用相同视觉元素，即使分开摆放也能保持整套产品的协调识别度。</x:v>
+        <x:v>🎁【圣诞袜礼物与派对赠礼】迷你小精灵可用作圣诞袜填充礼物、圣诞派对伴手礼及礼盒上的装饰。精灵服装和人物造型适合作为家人之间的圣诞小礼物，也适合喜欢收集迷你节日人物摆件的人。</x:v>
       </x:c>
       <x:c r="D8" s="40" t="str">
-        <x:v>开发文档 C3/F3；参考 B0CLJ8J4RP 图册02</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="285" customHeight="1">
+        <x:v>同款 B0CLJ8J4RP 第2、3、5点</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="390" customHeight="1">
       <x:c r="A9" s="39" t="str">
         <x:v>HTML 详情</x:v>
       </x:c>
       <x:c r="B9" s="40" t="str">
-        <x:v>&lt;p&gt;Quattro mini elfi di Natale in rosso, blu, verde e rosa aggiungono un accento coordinato alle composizioni dell’Avvento. Ogni statuina è alta circa 10,9 cm e dispone di braccia e gambe pieghevoli per cambiare posa.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Caratteristiche:&lt;/b&gt;&lt;br&gt;1. Quattro colori: un elfo rosso, uno blu, uno verde e uno rosa.&lt;br&gt;2. Presentazione flessibile: posa seduta, in piedi o inclinata.&lt;br&gt;3. Dettagli festivi: cappello a punta, colletto bianco, viso sorridente e scarpe rosse.&lt;br&gt;4. Uso versatile: albero, mensola, caminetto, tavola o pacco regalo.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Specifiche del prodotto:&lt;/b&gt;&lt;br&gt;Variante: set da 4&lt;br&gt;Altezza: circa 10,9 cm per statuina&lt;br&gt;Colori: rosso, blu, verde e rosa&lt;/p&gt;&lt;p&gt;&lt;b&gt;Contenuto della confezione:&lt;/b&gt;&lt;br&gt;4 × mini elfo di Natale&lt;/p&gt;</x:v>
+        <x:v>&lt;p&gt;Il set contiene quattro mini elfi di Natale, uno rosso, uno blu, uno verde e uno rosa. Ogni statuina è alta circa 10,9 cm e larga circa 5 cm, con braccia e gambe pieghevoli per decorazioni natalizie, storie con personaggi e piccoli regali.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Caratteristiche:&lt;/b&gt;&lt;br&gt;1. Quattro colori di abiti: I quattro elfi indossano tute rosse, blu, verdi e rosa con cappello a punta dello stesso colore. Il bordo del cappello, il pompon e il colletto a petali sono bianchi, mentre le scarpe sono rosse.&lt;br&gt;2. Arti pieghevoli: Le braccia possono essere alzate o rivolte ai lati e le gambe piegate in posizione seduta. È possibile anche una posizione in piedi per storie di elfi e giochi con personaggi natalizi.&lt;br&gt;3. Misure e dettagli: L’altezza dalla punta del cappello alla suola è di circa 10,9 cm, con una larghezza massima di circa 5 cm. Grandi occhi, sorriso, mani color carne, colletto bianco e scarpe rosse caratterizzano ogni statuina per camino, mensola o davanzale.&lt;br&gt;4. Decorazioni e piccoli doni: I personaggi sono adatti alle decorazioni natalizie accanto all’albero e sul tavolo, oltre che alle calze e ai pacchi regalo. Possono essere offerti durante le feste di Natale ai familiari o agli appassionati di piccole statuine stagionali.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Specifiche del prodotto:&lt;/b&gt;&lt;br&gt;Quantità: 4 statuine&lt;br&gt;Colori: 1 × rosso, blu, verde e rosa&lt;br&gt;Altezza totale per statuina: circa 10,9 cm&lt;br&gt;Larghezza massima per statuina: circa 5 cm&lt;br&gt;Struttura: braccia e gambe pieghevoli&lt;/p&gt;&lt;p&gt;&lt;b&gt;Contenuto della confezione:&lt;/b&gt;&lt;br&gt;4 × mini elfo di Natale, uno rosso, uno blu, uno verde e uno rosa&lt;/p&gt;</x:v>
       </x:c>
       <x:c r="C9" s="40" t="str">
-        <x:v>&lt;p&gt;红、蓝、绿、粉四色圣诞小精灵各1个，可为降临节和圣诞节陈列增加协调的节日色彩。单个约高10.9 cm，手臂和腿部可弯折，可按展示需要调整坐姿、站姿或其他姿态。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品特点：&lt;/b&gt;&lt;br&gt;1. 四色组合：红、蓝、绿、粉各1个，共4个。&lt;br&gt;2. 灵活摆放：可调整手脚姿态，适合不同陈列方式。&lt;br&gt;3. 节日造型：尖顶帽、白色领口、笑脸和红色鞋子。&lt;br&gt;4. 多种场景：适用于圣诞树、书架、壁炉架、桌面和礼品包装。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品参数：&lt;/b&gt;&lt;br&gt;规格：4件套&lt;br&gt;高度：单个约10.9 cm&lt;br&gt;颜色：红、蓝、绿、粉&lt;/p&gt;&lt;p&gt;&lt;b&gt;包装内容：&lt;/b&gt;&lt;br&gt;4 × 迷你圣诞小精灵&lt;/p&gt;</x:v>
+        <x:v>&lt;p&gt;这套迷你圣诞小精灵包含红、蓝、绿、粉四种颜色，各1个。单个约高10.9 cm、最宽约5 cm，手臂和双腿可弯折，适用于圣诞家居装饰、节日人物故事及小礼物。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品特点:&lt;/b&gt;&lt;br&gt;1. 四色服装: 四个小精灵分别穿红、蓝、绿、粉色连体服，尖顶帽与服装主色相配。帽檐、帽顶绒球和花瓣形领口为白色，鞋子为红色。&lt;br&gt;2. 可弯折四肢: 手臂可调整为抬起或位于身体两侧的姿势，双腿可弯曲呈坐姿。也可调整为站姿，用于圣诞小精灵故事和人物游戏。&lt;br&gt;3. 尺寸与外观: 从帽顶到鞋底总高约10.9 cm，最宽处约5 cm。大眼笑脸、肤色双手、白色领口和红色鞋子是每个小精灵的造型细节，可放在壁炉架、书架或窗台。&lt;br&gt;4. 节日装饰与赠礼: 可用作圣诞树旁和桌面的节日人物摆件，也可放入圣诞袜或作为礼盒装饰。适合作为圣诞派对小礼物，赠给家人或迷你节日人物收藏爱好者。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品参数:&lt;/b&gt;&lt;br&gt;数量：4个&lt;br&gt;颜色：红、蓝、绿、粉各1个&lt;br&gt;单个总高：约10.9 cm&lt;br&gt;单个最宽处：约5 cm&lt;br&gt;结构：手臂和双腿可弯折&lt;/p&gt;&lt;p&gt;&lt;b&gt;包装内容:&lt;/b&gt;&lt;br&gt;4 × 迷你圣诞小精灵，红、蓝、绿、粉各1个&lt;/p&gt;</x:v>
       </x:c>
       <x:c r="D9" s="40" t="str">
-        <x:v>开发文档 D3、C3/F3；参考 B0CLJ8J4RP 第1-5点</x:v>
+        <x:v>自有颜色、数量及图片；同款 B0CLJ8J4RP 第1–5点及尺寸图</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="75" customHeight="1">
@@ -1778,19 +1780,19 @@
         <x:v>Search Terms</x:v>
       </x:c>
       <x:c r="B10" s="40" t="str">
-        <x:v>gnometti soprammobili epifania calendario vetrina invernale bomboniera</x:v>
+        <x:v>gnometti folletti soprammobili calendario vetrina invernale bomboniera ornamento centrotavola gnomi tomte gonk addobbi vetrinistica segnaposto pupazzetti</x:v>
       </x:c>
       <x:c r="C10" s="40" t="str">
-        <x:v>小矮人 摆件 主显节 日历 冬季橱窗 宾客回礼</x:v>
+        <x:v>小矮人 小精灵 家居摆件 日历 橱窗 冬季 宾客回礼 饰品 餐桌中心装饰 地精 北欧地精 地精 节日装饰 橱窗陈列 座位标识 小玩偶</x:v>
       </x:c>
       <x:c r="D10" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP、B0CPJ65B1V 标题及五点/关键词提取</x:v>
+        <x:v>既有同款关键词候选及参考标题本地化；Amazon IT 本次页面访问受限，未声称当地搜索量</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31a850f934c947d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R315e52c06f534b54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1824,13 +1826,13 @@
         <x:v>Item Name</x:v>
       </x:c>
       <x:c r="B2" s="40" t="str">
-        <x:v>Pack de 4 mini elfos de Navidad, muñecos y figuras para Adviento</x:v>
+        <x:v>Pack de 4 mini elfos de Navidad, muñecos y figuras navideñas para Adviento</x:v>
       </x:c>
       <x:c r="C2" s="40" t="str">
-        <x:v>4个迷你圣诞小精灵，精灵玩偶和圣诞摆件，适用于降临节装饰。</x:v>
+        <x:v>4个迷你圣诞小精灵，精灵玩偶和圣诞摆件，适用于降临节布置。</x:v>
       </x:c>
       <x:c r="D2" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP、B0CPJ65B1V 标题；开发文档 D3</x:v>
+        <x:v>开发文档 D3；参考 B0CLJ8J4RP、B0CPJ65B1V 标题</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="71.25" customHeight="1">
@@ -1838,13 +1840,13 @@
         <x:v>Item Highlights</x:v>
       </x:c>
       <x:c r="B3" s="40" t="str">
-        <x:v>4 mini elfos rojo, azul, verde y rosa, aprox. 10,9 cm, flexibles para árbol, mesa, estante y decoración</x:v>
+        <x:v>4 mini elfos rojo, azul, verde y rosa, aprox. 10.9 cm, flexibles para árbol, mesa, estante, chimenea y decoración navideña</x:v>
       </x:c>
       <x:c r="C3" s="40" t="str">
-        <x:v>红、蓝、绿、粉四色迷你圣诞小精灵4件套，单个约10.9 cm，手脚可弯折摆姿，可用于圣诞树、桌面、置物架和降临节布置。</x:v>
+        <x:v>红、蓝、绿、粉四色迷你圣诞小精灵4件套，单个约高10.9 cm，手脚可弯折摆姿，可用于圣诞树、桌面、置物架、壁炉架和圣诞布置。</x:v>
       </x:c>
       <x:c r="D3" s="40" t="str">
-        <x:v>开发文档 D3、C3/F3；参考 B0CLJ8J4RP、B0CPJ65B1V</x:v>
+        <x:v>开发文档 D3、C3/F3；同款确认 I2/K2；参考 B0CLJ8J4RP、B0CPJ65B1V</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="165" customHeight="1">
@@ -1852,13 +1854,13 @@
         <x:v>五点 1</x:v>
       </x:c>
       <x:c r="B4" s="40" t="str">
-        <x:v>📦【Pack de cuatro colores】El paquete incluye cuatro mini elfos: uno rojo, uno azul, uno verde y uno rosa. La combinación definida facilita una composición coordinada y evita confundir los elementos de ambientación con el contenido real. Cada color aparece una sola vez, por lo que el contenido se reconoce de inmediato y las cuatro figuras pueden colocarse juntas o repartidas.</x:v>
+        <x:v>📦【Pack de 4 en rojo, azul, verde y rosa】El pack contiene cuatro mini elfos de Navidad: uno rojo, uno azul, uno verde y uno rosa. El gorro puntiagudo y el traje de cada personaje tienen el mismo color principal, con borde del gorro blanco, cuello blanco en forma de pétalos y zapatos rojos.</x:v>
       </x:c>
       <x:c r="C4" s="40" t="str">
-        <x:v>📦【四色4件套】包装内含4个迷你圣诞小精灵，红、蓝、绿、粉各1个。固定的四色组合便于形成协调陈列，也能让买家清楚区分实际包装内容与场景道具。每种颜色仅包含1个，四个产品既可以成组摆放，也可以分别布置在不同位置。</x:v>
+        <x:v>📦【红蓝绿粉四色套装】套装包含4个迷你圣诞小精灵，红色、蓝色、绿色和粉色各1个。每个小精灵的尖顶帽与连体服采用相同主色，搭配白色帽檐、白色花瓣领和红色鞋子。</x:v>
       </x:c>
       <x:c r="D4" s="40" t="str">
-        <x:v>开发文档 D3；参考 B0CPJ65B1V 第2点</x:v>
+        <x:v>开发表四色/件数；自有图片帽子和服装颜色</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="165" customHeight="1">
@@ -1866,13 +1868,13 @@
         <x:v>五点 2</x:v>
       </x:c>
       <x:c r="B5" s="40" t="str">
-        <x:v>🧩【Figuras articuladas】Cada elfo mide aproximadamente 10,9 cm y tiene brazos y piernas flexibles para colocarlo sentado, de pie o en otras posturas. Los muñecos elfo se adaptan así a distintas superficies decorativas. Los detalles repetidos crean una imagen coordinada, mientras que el rojo, azul, verde y rosa siguen siendo fáciles de distinguir dentro del conjunto.</x:v>
+        <x:v>🧩【Brazos y piernas flexibles】Los brazos y las piernas de los elfos se doblan para adoptar posturas sentadas, de pie o con los brazos levantados. Las piernas se flexionan hacia delante para sentarlos y los brazos pueden dirigirse hacia arriba o a los lados para representar personajes de historias navideñas.</x:v>
       </x:c>
       <x:c r="C5" s="40" t="str">
-        <x:v>🧩【可弯折造型】每个小精灵约高10.9 cm，手臂和腿部可弯折，可根据展示需要调整为坐姿、站姿或其他姿态。不同姿势便于适配桌面、置物架和节日布景；四款保持相同造型细节，仅以红、蓝、绿、粉颜色进行区分。</x:v>
+        <x:v>🧩【手臂与双腿可弯折】小精灵的手臂和双腿可以弯折，可调整为坐姿、站姿或抬手姿势。双腿向前弯曲可呈现坐姿，双臂可朝上或朝向身体两侧调整，用于圣诞小精灵故事中的角色动作。</x:v>
       </x:c>
       <x:c r="D5" s="40" t="str">
-        <x:v>同款确认 I2/K2；参考 B0CLJ8J4RP 第1点、B0CPJ65B1V 第3点</x:v>
+        <x:v>同款 B0CLJ8J4RP 第1、4点；四肢可弯折</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="165" customHeight="1">
@@ -1880,13 +1882,13 @@
         <x:v>五点 3</x:v>
       </x:c>
       <x:c r="B6" s="40" t="str">
-        <x:v>🎄【Decoración del árbol versátil】Coloca las figuras junto al árbol, en una estantería, sobre la chimenea o en el centro de una mesa festiva. Los cuatro colores pueden distribuirse por separado o reunirse como un pequeño conjunto. Así puedes formar un único punto focal o distribuir pequeños acentos navideños en distintas zonas de la habitación.</x:v>
+        <x:v>✨【Gorro con pompón y cara sonriente】Cada elfo tiene ojos grandes, una cara sonriente y manos y rostro de color carne. El gorro puntiagudo lleva borde y pompón blancos; una gola blanca en forma de pétalos remata la parte superior del traje, que cubre el torso y las piernas y termina en zapatos rojos.</x:v>
       </x:c>
       <x:c r="C6" s="40" t="str">
-        <x:v>🎄【多场景圣诞装饰】可将小精灵布置在圣诞树旁、壁炉架、书架、玄关柜或节日餐桌上。四种颜色既能集中形成完整视觉焦点，也能分散到房间不同区域，作为多个小型圣诞点缀，同时保持整套产品的统一感。</x:v>
+        <x:v>✨【尖帽绒球与笑脸造型】小精灵带有大眼睛、微笑表情和肤色面部及双手，尖顶帽配有白色帽檐和帽顶绒球。白色花瓣形领口围绕颈部，衣服覆盖躯干及双腿，脚部为红色鞋子造型。</x:v>
       </x:c>
       <x:c r="D6" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP 第1点和第5点</x:v>
+        <x:v>自有图片面部、帽子、领口、手部和鞋子</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="165" customHeight="1">
@@ -1894,13 +1896,13 @@
         <x:v>五点 4</x:v>
       </x:c>
       <x:c r="B7" s="40" t="str">
-        <x:v>🎁【Detalle de Adviento】Cada figura puede usarse como pequeña sorpresa, obsequio para invitados, relleno de calcetín o adorno para regalos. El pack se puede entregar completo o repartir entre varias personas. Las cuatro figuras también pueden repartirse entre varios paquetes, rincones de Adviento o composiciones de mesa según la presentación elegida.</x:v>
+        <x:v>📏【Tamaño mini de unos 10,9 cm】Cada figura mide aproximadamente 10,9 cm desde la punta del gorro hasta la suela de los zapatos y unos 5 cm en su parte más ancha. El tamaño mini sirve para decorar chimeneas, alféizares, librerías y mesas en Navidad, junto al árbol o en decoraciones de Adviento.</x:v>
       </x:c>
       <x:c r="C7" s="40" t="str">
-        <x:v>🎁【降临节小礼物】迷你小精灵可作为圣诞袜填充小礼物、派对伴手礼、礼品包装点缀或节日小惊喜。4个产品可以整套赠送，也可以分别搭配多个礼盒、降临节布置或桌面装饰，便于根据场景灵活安排。</x:v>
+        <x:v>📏【约10.9厘米迷你尺寸】每个小精灵从帽顶到鞋底总高约10.9 cm，最宽处约5 cm。迷你尺寸适用于壁炉架、窗台、书架和桌面的圣诞摆件，也可用于圣诞树旁及降临节装饰。</x:v>
       </x:c>
       <x:c r="D7" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP 第2、3、5点；B0CPJ65B1V 第4点</x:v>
+        <x:v>同款 B0CLJ8J4RP 尺寸图及第1点</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="165" customHeight="1">
@@ -1908,27 +1910,27 @@
         <x:v>五点 5</x:v>
       </x:c>
       <x:c r="B8" s="40" t="str">
-        <x:v>✨【Estilo de elfo coordinado】Los gorros puntiagudos, cuellos blancos, caras sonrientes y zapatos rojos dan a los cuatro personajes un aspecto uniforme. Su formato compacto encaja en espacios pequeños de decoración estacional. Los mismos elementos visuales se mantienen en los cuatro colores para que el conjunto siga reconociéndose como una colección coordinada.</x:v>
+        <x:v>🎁【Regalos para calcetines y fiestas】Los mini elfos se pueden incluir como regalos en calcetines navideños, ofrecer como detalles para invitados de una fiesta de Navidad o colocar sobre un paquete de regalo. Sus trajes de elfo los convierten en pequeños regalos navideños para familiares y aficionados a coleccionar figuras miniatura de temporada.</x:v>
       </x:c>
       <x:c r="C8" s="40" t="str">
-        <x:v>✨【统一精灵造型】尖顶帽、白色帽檐与绒球、白色花瓣形领口、笑脸和红色鞋子，让四个小精灵形成一致的节日造型。红、蓝、绿、粉四款沿用相同视觉元素，即使分开摆放也能保持整套产品的协调识别度。</x:v>
+        <x:v>🎁【圣诞袜礼物与派对赠礼】迷你小精灵可用作圣诞袜填充礼物、圣诞派对伴手礼及礼盒上的装饰。精灵服装和人物造型适合作为家人之间的圣诞小礼物，也适合喜欢收集迷你节日人物摆件的人。</x:v>
       </x:c>
       <x:c r="D8" s="40" t="str">
-        <x:v>开发文档 C3/F3；参考 B0CLJ8J4RP 图册02</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="285" customHeight="1">
+        <x:v>同款 B0CLJ8J4RP 第2、3、5点</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="390" customHeight="1">
       <x:c r="A9" s="39" t="str">
         <x:v>HTML 详情</x:v>
       </x:c>
       <x:c r="B9" s="40" t="str">
-        <x:v>&lt;p&gt;Cuatro mini elfos en rojo, azul, verde y rosa aportan un toque coordinado a los ambientes de Adviento y Navidad. Cada figura mide aproximadamente 10,9 cm y dispone de brazos y piernas flexibles para cambiar de postura.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Características:&lt;/b&gt;&lt;br&gt;1. Cuatro colores: un elfo rojo, uno azul, uno verde y uno rosa.&lt;br&gt;2. Presentación flexible: postura sentada, de pie o inclinada.&lt;br&gt;3. Detalles festivos: gorro puntiagudo, cuello blanco, cara sonriente y zapatos rojos.&lt;br&gt;4. Uso versátil: árbol, estantería, chimenea, mesa o paquete de regalo.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Especificaciones del producto:&lt;/b&gt;&lt;br&gt;Variante: pack de 4&lt;br&gt;Altura: aproximadamente 10,9 cm por figura&lt;br&gt;Colores: rojo, azul, verde y rosa&lt;/p&gt;&lt;p&gt;&lt;b&gt;Contenido del paquete:&lt;/b&gt;&lt;br&gt;4 × mini elfo&lt;/p&gt;</x:v>
+        <x:v>&lt;p&gt;El pack incluye cuatro mini elfos de Navidad, uno rojo, uno azul, uno verde y uno rosa. Cada figura mide aproximadamente 10,9 cm de alto y 5 cm de ancho, con brazos y piernas flexibles para decorar en Navidad, representar historias y ofrecer pequeños regalos.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Características:&lt;/b&gt;&lt;br&gt;1. Trajes de cuatro colores: Los cuatro elfos llevan trajes rojos, azules, verdes y rosas con un gorro puntiagudo del mismo color. El borde del gorro, el pompón y el cuello en forma de pétalos son blancos, mientras que los zapatos son rojos.&lt;br&gt;2. Extremidades flexibles: Los brazos se pueden levantar o dirigir hacia los lados y las piernas se doblan para adoptar una postura sentada. También pueden adoptar una postura de pie para historias de elfos y juegos con personajes de Navidad.&lt;br&gt;3. Medidas y detalles: La altura desde la punta del gorro hasta la suela es de unos 10,9 cm, con aproximadamente 5 cm de anchura máxima. Ojos grandes, sonrisa, manos de color carne, cuello blanco y zapatos rojos forman cada figura para chimeneas, estantes o alféizares.&lt;br&gt;4. Decoración y pequeños regalos: Los personajes sirven como adornos navideños junto al árbol y en la mesa, además de regalos para calcetines o decoración de paquetes. Se pueden ofrecer como detalles en fiestas de Navidad a familiares o a aficionados a las pequeñas figuras de temporada.&lt;/p&gt;&lt;p&gt;&lt;b&gt;Especificaciones del producto:&lt;/b&gt;&lt;br&gt;Cantidad: 4 figuras&lt;br&gt;Colores: 1 × rojo, azul, verde y rosa&lt;br&gt;Altura total por figura: unos 10,9 cm&lt;br&gt;Anchura máxima por figura: unos 5 cm&lt;br&gt;Estructura: brazos y piernas flexibles&lt;/p&gt;&lt;p&gt;&lt;b&gt;Contenido del paquete:&lt;/b&gt;&lt;br&gt;4 × mini elfo de Navidad, uno rojo, uno azul, uno verde y uno rosa&lt;/p&gt;</x:v>
       </x:c>
       <x:c r="C9" s="40" t="str">
-        <x:v>&lt;p&gt;红、蓝、绿、粉四色圣诞小精灵各1个，可为降临节和圣诞节陈列增加协调的节日色彩。单个约高10.9 cm，手臂和腿部可弯折，可按展示需要调整坐姿、站姿或其他姿态。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品特点：&lt;/b&gt;&lt;br&gt;1. 四色组合：红、蓝、绿、粉各1个，共4个。&lt;br&gt;2. 灵活摆放：可调整手脚姿态，适合不同陈列方式。&lt;br&gt;3. 节日造型：尖顶帽、白色领口、笑脸和红色鞋子。&lt;br&gt;4. 多种场景：适用于圣诞树、书架、壁炉架、桌面和礼品包装。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品参数：&lt;/b&gt;&lt;br&gt;规格：4件套&lt;br&gt;高度：单个约10.9 cm&lt;br&gt;颜色：红、蓝、绿、粉&lt;/p&gt;&lt;p&gt;&lt;b&gt;包装内容：&lt;/b&gt;&lt;br&gt;4 × 迷你圣诞小精灵&lt;/p&gt;</x:v>
+        <x:v>&lt;p&gt;这套迷你圣诞小精灵包含红、蓝、绿、粉四种颜色，各1个。单个约高10.9 cm、最宽约5 cm，手臂和双腿可弯折，适用于圣诞家居装饰、节日人物故事及小礼物。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品特点:&lt;/b&gt;&lt;br&gt;1. 四色服装: 四个小精灵分别穿红、蓝、绿、粉色连体服，尖顶帽与服装主色相配。帽檐、帽顶绒球和花瓣形领口为白色，鞋子为红色。&lt;br&gt;2. 可弯折四肢: 手臂可调整为抬起或位于身体两侧的姿势，双腿可弯曲呈坐姿。也可调整为站姿，用于圣诞小精灵故事和人物游戏。&lt;br&gt;3. 尺寸与外观: 从帽顶到鞋底总高约10.9 cm，最宽处约5 cm。大眼笑脸、肤色双手、白色领口和红色鞋子是每个小精灵的造型细节，可放在壁炉架、书架或窗台。&lt;br&gt;4. 节日装饰与赠礼: 可用作圣诞树旁和桌面的节日人物摆件，也可放入圣诞袜或作为礼盒装饰。适合作为圣诞派对小礼物，赠给家人或迷你节日人物收藏爱好者。&lt;/p&gt;&lt;p&gt;&lt;b&gt;产品参数:&lt;/b&gt;&lt;br&gt;数量：4个&lt;br&gt;颜色：红、蓝、绿、粉各1个&lt;br&gt;单个总高：约10.9 cm&lt;br&gt;单个最宽处：约5 cm&lt;br&gt;结构：手臂和双腿可弯折&lt;/p&gt;&lt;p&gt;&lt;b&gt;包装内容:&lt;/b&gt;&lt;br&gt;4 × 迷你圣诞小精灵，红、蓝、绿、粉各1个&lt;/p&gt;</x:v>
       </x:c>
       <x:c r="D9" s="40" t="str">
-        <x:v>开发文档 D3、C3/F3；参考 B0CLJ8J4RP 第1-5点</x:v>
+        <x:v>自有颜色、数量及图片；同款 B0CLJ8J4RP 第1–5点及尺寸图</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="75" customHeight="1">
@@ -1936,19 +1938,19 @@
         <x:v>Search Terms</x:v>
       </x:c>
       <x:c r="B10" s="40" t="str">
-        <x:v>duendecillos bibelots escaparate invernal calendario aguinaldo</x:v>
+        <x:v>duendecillos gnomos enanos gonk estatuitas escaparate invernal calendario aguinaldo miniaturas sobremesa tomte duendes suecos figuritas muñequitos ornamentos repisa escaparates pueblo</x:v>
       </x:c>
       <x:c r="C10" s="40" t="str">
-        <x:v>圣诞小矮人 摆件 降临节日历 礼袋填充物 冬季橱窗</x:v>
+        <x:v>小精灵 地精 小矮人 北欧地精 小雕像 橱窗 冬季 日历 圣诞小礼物 微缩模型 桌面摆件 北欧地精 小妖精 瑞典的 小摆件 小玩偶 饰品 置物架 橱窗 村庄</x:v>
       </x:c>
       <x:c r="D10" s="40" t="str">
-        <x:v>参考 B0CLJ8J4RP、B0CPJ65B1V 标题及五点/关键词提取</x:v>
+        <x:v>既有同款关键词候选；Amazon ES“duendecillos gnomos navidad figuras”前20个结果复核；参考标题</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb28d1786058043d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20bdd5301ca04ca5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>